<commit_message>
fix: resolve merge conflict in index.js, add CSS imports
Keeps ThemeProvider/CssBaseline setup from main, adds missing
index.css and App.css imports for Tailwind styles.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vyuziti bezpecnostnich opatreni.xlsx
+++ b/Vyuziti bezpecnostnich opatreni.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zk/event-security-planner/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zk/STW/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FCB2EE2-E555-B24D-B8C5-9867FFF59E70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A78A5BF-299E-6F41-8532-5F63F1DDD70B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="160" yWindow="920" windowWidth="29080" windowHeight="14480" xr2:uid="{9E7D9EB1-F9C1-5243-8C6E-597A7DCF73BC}"/>
   </bookViews>
@@ -587,6 +587,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6799597-7DDE-2C4D-9160-A8764E141969}">
   <dimension ref="A1:W20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="23.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="80" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>

</xml_diff>